<commit_message>
Add ranked recommendation and fill workbook decision cells
- results/recommendation.json: ranked recommendation (distilled student
  first) with verdicts, rationale and residual risks from the T4 run
- build_workbook.py reads it to fill Board Rank/Verdict and the
  Recommendation sheet, so rebuilds keep the ranking
- Rebuilt brightline_benchmark.xlsx from the T4 runs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/brightline_benchmark.xlsx
+++ b/results/brightline_benchmark.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Board" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Runs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Training" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scaling" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommendation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Board" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Runs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Training" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scaling" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Recommendation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Protocol" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -156,7 +156,9 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,9 +181,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -289,14 +289,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -317,7 +317,7 @@
             <v>baseline</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -326,10 +326,10 @@
             <symbol val="circle"/>
             <size val="11"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="2F5597"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:solidFill>
                   <a:srgbClr val="2F5597"/>
                 </a:solidFill>
@@ -355,7 +355,7 @@
             <v>linear_attention</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -364,10 +364,10 @@
             <symbol val="circle"/>
             <size val="11"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="ED7D31"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:solidFill>
                   <a:srgbClr val="ED7D31"/>
                 </a:solidFill>
@@ -393,7 +393,7 @@
             <v>quant_4bit</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -402,10 +402,10 @@
             <symbol val="circle"/>
             <size val="11"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="70AD47"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:solidFill>
                   <a:srgbClr val="70AD47"/>
                 </a:solidFill>
@@ -431,7 +431,7 @@
             <v>distilled_student</v>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -440,10 +440,10 @@
             <symbol val="circle"/>
             <size val="11"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="7030A0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:solidFill>
                   <a:srgbClr val="7030A0"/>
                 </a:solidFill>
@@ -475,8 +475,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -503,8 +503,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -532,14 +532,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -564,10 +564,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="2F5597"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -733,7 +733,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -748,9 +748,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -770,9 +770,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1127,7 +1127,7 @@
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="7" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="48" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1373,8 +1373,14 @@
         <f>IF(F12="","",IF(AND(F12&gt;=$B$7,J12&lt;=$B$8,M12&lt;=$B$9),"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="S12" s="20" t="n"/>
-      <c r="T12" s="21" t="n"/>
+      <c r="S12" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="T12" s="21" t="inlineStr">
+        <is>
+          <t>Reference only. Accurate, but the largest download and memory footprint.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1453,8 +1459,14 @@
         <f>IF(F13="","",IF(AND(F13&gt;=$B$7,J13&lt;=$B$8,M13&lt;=$B$9),"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="S13" s="20" t="n"/>
-      <c r="T13" s="21" t="n"/>
+      <c r="S13" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="T13" s="21" t="inlineStr">
+        <is>
+          <t>Do not ship. Slower and less accurate at our input lengths.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1533,8 +1545,14 @@
         <f>IF(F14="","",IF(AND(F14&gt;=$B$7,J14&lt;=$B$8,M14&lt;=$B$9),"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="S14" s="20" t="n"/>
-      <c r="T14" s="21" t="n"/>
+      <c r="S14" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="T14" s="21" t="inlineStr">
+        <is>
+          <t>Runner-up. No accuracy loss and 4.6x smaller, but 2x slower on GPU and the tablet runtime is unproven.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1613,8 +1631,14 @@
         <f>IF(F15="","",IF(AND(F15&gt;=$B$7,J15&lt;=$B$8,M15&lt;=$B$9),"PASS","FAIL"))</f>
         <v/>
       </c>
-      <c r="S15" s="20" t="n"/>
-      <c r="T15" s="21" t="n"/>
+      <c r="S15" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" s="21" t="inlineStr">
+        <is>
+          <t>SHIP. Same accuracy within noise, fastest, smallest, half the memory.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -4644,7 +4668,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in after the Colab run. Rank 1 is the configuration to ship; ranks should match Board!S.</t>
+          <t>Rank 1 is the configuration to ship. Edit results/recommendation.json and rebuild to change it.</t>
         </is>
       </c>
     </row>
@@ -4685,11 +4709,15 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="66" customHeight="1">
       <c r="A5" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="21" t="n"/>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>distilled_student</t>
+        </is>
+      </c>
       <c r="C5" s="13">
         <f>IF(B5="","",INDEX(Board!$F$12:$F$15,MATCH(B5,Board!$A$12:$A$15,0)))</f>
         <v/>
@@ -4702,14 +4730,26 @@
         <f>IF(B5="","",INDEX(Board!$M$12:$M$15,MATCH(B5,Board!$A$12:$A$15,0)))</f>
         <v/>
       </c>
-      <c r="F5" s="40" t="n"/>
-      <c r="G5" s="40" t="n"/>
-    </row>
-    <row r="6">
+      <c r="F5" s="21" t="inlineStr">
+        <is>
+          <t>-0.3 pts accuracy (7 of 2,493 test items, inside the ~0.65-pt standard error) for 1.6x faster p95 (mean of trials), 6.2x smaller download and half the peak memory of the baseline.</t>
+        </is>
+      </c>
+      <c r="G5" s="21" t="inlineStr">
+        <is>
+          <t>Driver-note accuracy is 72.7%, so roughly 1 in 4 spoken notes is misrouted unless the driver confirms it. Latency was measured on a T4 GPU, not the tablet. Document accuracy is on synthetic scans.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
       <c r="A6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="21" t="n"/>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>quant_4bit</t>
+        </is>
+      </c>
       <c r="C6" s="13">
         <f>IF(B6="","",INDEX(Board!$F$12:$F$15,MATCH(B6,Board!$A$12:$A$15,0)))</f>
         <v/>
@@ -4722,14 +4762,26 @@
         <f>IF(B6="","",INDEX(Board!$M$12:$M$15,MATCH(B6,Board!$A$12:$A$15,0)))</f>
         <v/>
       </c>
-      <c r="F6" s="40" t="n"/>
-      <c r="G6" s="40" t="n"/>
-    </row>
-    <row r="7">
+      <c r="F6" s="21" t="inlineStr">
+        <is>
+          <t>Matches baseline accuracy at 4.6x smaller, but bitsandbytes 4-bit is CUDA-only and unpacking weights makes single requests ~2x slower on the T4.</t>
+        </is>
+      </c>
+      <c r="G6" s="21" t="inlineStr">
+        <is>
+          <t>Needs a different int4 runtime on Android whose speed and accuracy are unmeasured; the GPU latency result may not carry over in either direction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
       <c r="A7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="21" t="n"/>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>baseline</t>
+        </is>
+      </c>
       <c r="C7" s="13">
         <f>IF(B7="","",INDEX(Board!$F$12:$F$15,MATCH(B7,Board!$A$12:$A$15,0)))</f>
         <v/>
@@ -4742,14 +4794,26 @@
         <f>IF(B7="","",INDEX(Board!$M$12:$M$15,MATCH(B7,Board!$A$12:$A$15,0)))</f>
         <v/>
       </c>
-      <c r="F7" s="40" t="n"/>
-      <c r="G7" s="40" t="n"/>
-    </row>
-    <row r="8">
+      <c r="F7" s="21" t="inlineStr">
+        <is>
+          <t>Best-in-class accuracy alongside 4-bit, but 13.3 MB and 30 MB peak memory buy nothing over the student.</t>
+        </is>
+      </c>
+      <c r="G7" s="21" t="inlineStr">
+        <is>
+          <t>Largest OTA update and memory footprint on the tablet for no measurable accuracy gain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
       <c r="A8" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="21" t="n"/>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>linear_attention</t>
+        </is>
+      </c>
       <c r="C8" s="13">
         <f>IF(B8="","",INDEX(Board!$F$12:$F$15,MATCH(B8,Board!$A$12:$A$15,0)))</f>
         <v/>
@@ -4762,8 +4826,16 @@
         <f>IF(B8="","",INDEX(Board!$M$12:$M$15,MATCH(B8,Board!$A$12:$A$15,0)))</f>
         <v/>
       </c>
-      <c r="F8" s="40" t="n"/>
-      <c r="G8" s="40" t="n"/>
+      <c r="F8" s="21" t="inlineStr">
+        <is>
+          <t>-1.0 pts accuracy (-3.0 pts on notes) and 1.6x slower p95: at ~160 tokens per request, linear attention's O(T) advantage never materializes.</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="inlineStr">
+        <is>
+          <t>Would only pay off for much longer inputs (multi-page documents), which we have not benchmarked.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">

</xml_diff>